<commit_message>
Add BIN payload type with octet-stream transmission
</commit_message>
<xml_diff>
--- a/samples/config-all-cases.xlsx
+++ b/samples/config-all-cases.xlsx
@@ -10,14 +10,14 @@
     <sheet name="PayloadTypes" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Settings!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">PayloadTypes!$A$1:$E$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Settings!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">PayloadTypes!$A$1:$F$121</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="37">
   <si>
     <t>key</t>
   </si>
@@ -64,6 +64,15 @@
     <t>[]</t>
   </si>
   <si>
+    <t>headers</t>
+  </si>
+  <si>
+    <t>{}</t>
+  </si>
+  <si>
+    <t>payloadSizes</t>
+  </si>
+  <si>
     <t>contentType</t>
   </si>
   <si>
@@ -116,6 +125,9 @@
   </si>
   <si>
     <t>multipart</t>
+  </si>
+  <si>
+    <t>bin</t>
   </si>
 </sst>
 </file>
@@ -184,7 +196,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="30.0" customWidth="true"/>
@@ -255,15 +267,31 @@
         <v>14</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B8"/>
+  <autoFilter ref="A1:B10"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E97"/>
+  <dimension ref="A1:F121"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="26.0" customWidth="true"/>
@@ -271,17 +299,18 @@
     <col min="3" max="3" width="26.0" customWidth="true"/>
     <col min="4" max="4" width="26.0" customWidth="true"/>
     <col min="5" max="5" width="26.0" customWidth="true"/>
+    <col min="6" max="6" width="26.0" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1" ht="24.0" customHeight="true">
       <c r="A1" t="s" s="2">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B1" t="s" s="2">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C1" t="s" s="2">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D1" t="s" s="2">
         <v>8</v>
@@ -289,1065 +318,1692 @@
       <c r="E1" t="s" s="2">
         <v>10</v>
       </c>
+      <c r="F1" t="s" s="2">
+        <v>15</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F11" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F12" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F13" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F14" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F15" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F16" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F17" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C18" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F18" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C19" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F19" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C20" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F20" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C21" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F21" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C22" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F22" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C23" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F23" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C24" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F24" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C25" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F25" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C26" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F26" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C27" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F27" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C28" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F28" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C29" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F29" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C30" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F30" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C31" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F31" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C32" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F32" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C33" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F33" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C34" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F34" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C35" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F35" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C36" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F36" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C37" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F37" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C38" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F38" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C39" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F39" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C40" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F40" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B41" t="s" s="0">
         <v>30</v>
       </c>
-      <c r="B41" t="s" s="0">
-        <v>27</v>
-      </c>
       <c r="C41" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F41" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B42" t="s" s="0">
         <v>30</v>
       </c>
-      <c r="B42" t="s" s="0">
-        <v>27</v>
-      </c>
       <c r="C42" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F42" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B43" t="s" s="0">
         <v>30</v>
       </c>
-      <c r="B43" t="s" s="0">
-        <v>27</v>
-      </c>
       <c r="C43" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F43" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C44" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F44" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C45" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F45" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C46" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F46" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C47" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F47" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C48" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F48" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C49" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F49" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C50" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F50" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C51" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F51" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C52" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F52" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C53" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F53" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C54" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F54" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C55" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F55" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C56" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F56" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C57" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F57" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B58" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C58" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F58" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C59" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F59" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B60" t="s" s="0">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C60" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F60" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C61" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F61" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B62" t="s" s="0">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C62" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F62" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B63" t="s" s="0">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C63" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F63" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B64" t="s" s="0">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C64" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F64" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B65" t="s" s="0">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C65" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F65" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B66" t="s" s="0">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C66" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F66" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B67" t="s" s="0">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C67" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F67" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B68" t="s" s="0">
         <v>31</v>
       </c>
-      <c r="B68" t="s" s="0">
-        <v>28</v>
-      </c>
       <c r="C68" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F68" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B69" t="s" s="0">
         <v>31</v>
       </c>
-      <c r="B69" t="s" s="0">
-        <v>28</v>
-      </c>
       <c r="C69" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F69" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B70" t="s" s="0">
         <v>31</v>
       </c>
-      <c r="B70" t="s" s="0">
-        <v>28</v>
-      </c>
       <c r="C70" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F70" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B71" t="s" s="0">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C71" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F71" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B72" t="s" s="0">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C72" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F72" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B73" t="s" s="0">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C73" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F73" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B74" t="s" s="0">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C74" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F74" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B75" t="s" s="0">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C75" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F75" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B76" t="s" s="0">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C76" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F76" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B77" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C77" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F77" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B78" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C78" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F78" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B79" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C79" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F79" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B80" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C80" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F80" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B81" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C81" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F81" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B82" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C82" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F82" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B83" t="s" s="0">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C83" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F83" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B84" t="s" s="0">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C84" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F84" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B85" t="s" s="0">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C85" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F85" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B86" t="s" s="0">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C86" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F86" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B87" t="s" s="0">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C87" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F87" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B88" t="s" s="0">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C88" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F88" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B89" t="s" s="0">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C89" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F89" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B90" t="s" s="0">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C90" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F90" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B91" t="s" s="0">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C91" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F91" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B92" t="s" s="0">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C92" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F92" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B93" t="s" s="0">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C93" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F93" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B94" t="s" s="0">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C94" t="s" s="0">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="F94" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B95" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="B95" t="s" s="0">
-        <v>29</v>
-      </c>
       <c r="C95" t="s" s="0">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="F95" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B96" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="B96" t="s" s="0">
-        <v>29</v>
-      </c>
       <c r="C96" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="F96" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B97" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="B97" t="s" s="0">
+      <c r="C97" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="F97" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B98" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C98" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F98" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B99" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C99" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="F99" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B100" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C100" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="F100" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B101" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="C101" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F101" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B102" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="C102" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="F102" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B103" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="C103" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="F103" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B104" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C104" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F104" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B105" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C105" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="F105" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B106" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C106" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="F106" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B107" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C107" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F107" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B108" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C108" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="F108" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B109" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C109" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="F109" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B110" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="C97" t="s" s="0">
-        <v>22</v>
+      <c r="C110" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F110" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B111" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="C111" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="F111" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B112" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="C112" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="F112" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B113" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="C113" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F113" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B114" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="C114" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="F114" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B115" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="C115" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="F115" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B116" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="C116" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F116" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B117" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="C117" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="F117" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B118" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="C118" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="F118" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B119" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="C119" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="F119" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B120" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="C120" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="F120" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B121" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="C121" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="F121" t="s" s="0">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E97"/>
+  <autoFilter ref="A1:F121"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>